<commit_message>
Taking a new export of the words
</commit_message>
<xml_diff>
--- a/exports/excel/vocabulary_id.xlsx
+++ b/exports/excel/vocabulary_id.xlsx
@@ -413,14 +413,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F253"/>
+  <dimension ref="A1:F380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -8004,6 +8004,3816 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Klavier</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Piano</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Klaviere</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Rad</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Bike</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Räder</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Kino</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Cinema</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Kinos</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Park</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Park</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Parke</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Computerspiel</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Computer Game</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Computerspiele</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Spaß</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Fun</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Späße</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Stresse</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Free Time</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Freizeiten</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Disco</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Discos</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Tage</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Montage</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Dienstag</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Dienstage</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Mittwoch</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Mittwoche</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Donnerstag</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Donnerstage</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Freitag</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Freitage</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Samstag</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Samstage</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Sonntag</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Sonntage</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Konzert</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Concert</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Konzerte</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Theater</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Theater</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Theater</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Leser</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Reader (M)</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Leser</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Leserin</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Reader (F)</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Leserinnen</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Kreis</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Circle</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Kreise</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Gedicht</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Poem</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Gedichte</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Idee</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Ideen</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Wohnung</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Apartment</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Wohnungen</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Arbeitsplatz</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Workplace</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Arbeitsplätze</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Notfall</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Notfälle</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Arzt</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Doctor (M)</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Ärzte</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Ärztin</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Doctor (F)</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Ärztinnen</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Krankenpfleger</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Nurse (M)</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Krankenpfleger</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Krankenpflegering</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Nurse (F)</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Krankenpflegerinnen</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Krankenschwester</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Nurse</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Krankenschwester</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Krankenhaus</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Krankenhäuser</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Tankstelle</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Gas Station</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Tankstellen</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Flughafen</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Flughäfen</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Bahnhof</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Train Station</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Bahnhöfe</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Geschäft</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Geschäfte</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Schule</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Sculen</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Kirche</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Church</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Kirchen</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Lücke</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Lücken</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Zentrum</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Center</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Zentren</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Tiergarten</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Zoo</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Tiergärten</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Stadtpark</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>City Park</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Stadtparke</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Dorf</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Village</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Dörfer</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Miete</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Mieten</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Traum</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Dream</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Träume</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Pinnwand</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Bulletin Board</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Pinnwände</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Wahl</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Vote</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Wahlen</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Zimmer</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Room</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Zimmer</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Wohngemeinschaft</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Shared Apartment</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Wohngemeinschaften</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Parkbank</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Park Bench</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Parkbanken</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Möbeln</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Fernseher</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Television</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Fernseher</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Schrank</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Closet</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Schränke</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Bett</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Bed</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Betten</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Kühlschrank</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Kühlschränke</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Mikrowelle</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Microwave</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Mikrowellen</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Lampe</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Lamp</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Lampen</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Klosett</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Toilet</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Klosette</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Couch</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Couch</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Couchen</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Wohnzimmer</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Living Room</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Wohnzimmer</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Schlafzimmer</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Bedroom</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Schlafzimmer</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Bad</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Bäder</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Balkon</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Balcony</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Balkone</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Mitte</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Mitten</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Dunkel</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Darkness</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Dunkels</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Luxus</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Luxus</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Gastzimmer</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Guest Room</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Gastzimmer</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Bäckerei</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Bakery</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Bäckereien</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Etage</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Etagen</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>323</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Sonne</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Sonnen</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>324</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Regen</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Rain</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Regen</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>325</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Schnee</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Snow</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Schnees</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>326</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Wolke</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Wolken</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>327</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Temperatur</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Temperaturen</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>328</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>329</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Wettervorhersage</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Weather forecast</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Wettervorhersagen</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>330</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Wetter</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Wetter</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>331</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Morgen</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Morgen</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>332</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Vormittag</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Forenoon</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Vormittage</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>333</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Mittag</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Noon</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Mittage</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>334</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Nachmittag</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Nachmittage</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Abend</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Abende</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Nacht</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Night</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Nächte</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Norden</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Nordens</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Süden</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Südens</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Westen</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Westens</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Osten</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Ostens</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Fahrradkurier</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Bicycle Courier</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Fahrradkuriere</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Autobahn</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Highway</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Autobahnen</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Geburt</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Birth</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Geburten</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Geburtsort</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Birthplace</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Geburtsorte</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Geburtsdatum</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Date of Birth</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Geburtsdatumen</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Geburtstag</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Geburtstage</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Universität</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Universitäten</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Praktikant</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Praktikanten</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Lebenslauf</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Lebensläufe</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Fremdsprache</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Foreign Language</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Fremdsprachen</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Orte</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Abitur</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Abitur</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Abiture</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Matura</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>High school diploma</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Matura</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Zug</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Train</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Züge</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Umwelt</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Umwelten</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Flugzeug</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Airplane</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Flugzeuge</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Stau</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Traffic Jam</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Staus</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Verkehr</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Traffic</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Verkehre</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Verkehrsmittel</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Means of Transportation</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Verkehrsmittel</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Bushaltestelle</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Bus Stop</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Bushaltestellen</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Straßembahn</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Tram</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Straßembahnen</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Metros</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Würfel</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Würfel</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Gleis</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Gleise</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Abfahrt</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Abfahrten</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Einwohner</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Resident (M)</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Einwohner</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Einwohnerin</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Resident (F)</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Einwohnerinnen</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Sehenswürdigkeit</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Sight</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Sehenswürdigkeiten</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Hexe</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Witch</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Hexen</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Vampir</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Vampire (M)</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Vampire</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Vampirin</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Vampire (F)</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Vampirinnen</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Treffpunkt</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Meeting Point</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Treffpunkte</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Geheimnis</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Geheimnisse</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Gasse</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>die</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Alley</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Gassen</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Rathaus</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>City Hall</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Rathäuser</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Marktplatz</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Marktplätze</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Pfeil</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Arrow</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Pfeile</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Schloss</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Palace</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Schlösser</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Strand</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>der</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Beach</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Strände</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>